<commit_message>
K10 report vzhled OK
</commit_message>
<xml_diff>
--- a/admin_testy/reporty_google_testy/google_data/Pobočky/Prosek/Report Prosek.xlsx
+++ b/admin_testy/reporty_google_testy/google_data/Pobočky/Prosek/Report Prosek.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1939" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1949" uniqueCount="717">
   <si>
     <t>Datum</t>
   </si>
@@ -1929,7 +1929,7 @@
     <t>Makula Radek</t>
   </si>
   <si>
-    <t>38:00</t>
+    <t>52:00</t>
   </si>
   <si>
     <t>29:00</t>
@@ -1938,34 +1938,61 @@
     <t>Vychivskyi Volodymyr</t>
   </si>
   <si>
-    <t>63:00</t>
+    <t>120:00</t>
   </si>
   <si>
     <t>Šebesta Tomáš</t>
   </si>
   <si>
+    <t>56:00</t>
+  </si>
+  <si>
     <t>23:00</t>
   </si>
   <si>
     <t>Kačena Stanislav</t>
   </si>
   <si>
-    <t>6:00</t>
+    <t>19:00</t>
   </si>
   <si>
     <t>Nováková Adéla</t>
   </si>
   <si>
-    <t>69:00</t>
+    <t>133:00</t>
   </si>
   <si>
     <t>13:00</t>
   </si>
   <si>
+    <t>Hanibal Filip</t>
+  </si>
+  <si>
+    <t>8:00</t>
+  </si>
+  <si>
+    <t>Kopic Jakub</t>
+  </si>
+  <si>
+    <t>22:30</t>
+  </si>
+  <si>
+    <t>Putna Jaroslav</t>
+  </si>
+  <si>
     <t>7:00</t>
   </si>
   <si>
-    <t>11 min 02 s</t>
+    <t>Ahurieva Viktoriia</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>Gorol Patrik</t>
+  </si>
+  <si>
+    <t>11 min 50 s</t>
   </si>
   <si>
     <t>Manažeři</t>
@@ -13244,7 +13271,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="9">
-        <v>46154.0</v>
+        <v>46162.0</v>
       </c>
       <c r="E1" s="10"/>
       <c r="F1" s="11" t="s">
@@ -13293,7 +13320,7 @@
       <c r="A3" s="24"/>
       <c r="B3" s="25" t="str">
         <f>CHOOSE(WEEKDAY(D1), "Neděle", "Pondělí", "Úterý", "Středa", "Čtvrtek", "Pátek", "Sobota")</f>
-        <v>Úterý</v>
+        <v>Středa</v>
       </c>
       <c r="C3" s="26"/>
       <c r="D3" s="26"/>
@@ -13804,7 +13831,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I26" s="86">
         <f t="shared" si="3"/>
@@ -13845,7 +13872,7 @@
         <v>0</v>
       </c>
       <c r="H27" s="82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" s="86">
         <f t="shared" si="3"/>
@@ -14081,7 +14108,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" sqref="B12:B21">
-      <formula1>"Nedbal Michal,Ahurieva Viktoriia,Pešová Hana,Šebesta Tomáš,Nováková Adéla,Makula Radek,Putna Jaroslav,Kopic Jakub,Fáberová Kateřina"</formula1>
+      <formula1>"Nedbal Michal,Ahurieva Viktoriia,Pešová Hana,Šebesta Tomáš,Coufal Jakub,Nováková Adéla,Makula Radek,Gorol Patrik,Putna Jaroslav,Kopic Jakub,Fáberová Kateřina"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B25:B31">
       <formula1>"Hanibal Filip,Mikuš Pavel,Šmídová Sabina,Kormash Liubov,Vychivskyi Volodymyr,Hřebík Martin,Reischl Jan,Kulinič Michail,Kačena Stanislav"</formula1>
@@ -14121,7 +14148,7 @@
         <v>631</v>
       </c>
       <c r="E1" s="109">
-        <v>46173.0</v>
+        <v>46160.0</v>
       </c>
       <c r="F1" s="110" t="s">
         <v>586</v>
@@ -14146,18 +14173,18 @@
       <c r="D2" s="16"/>
       <c r="E2" s="18"/>
       <c r="F2" s="112">
-        <v>0.32496139858532447</v>
+        <v>0.34210884172421985</v>
       </c>
       <c r="H2" s="20"/>
       <c r="I2" s="113">
-        <v>270705.0</v>
+        <v>570148.7999999999</v>
       </c>
       <c r="K2" s="20"/>
       <c r="L2" s="114" t="s">
         <v>589</v>
       </c>
       <c r="M2" s="115">
-        <v>97298.0</v>
+        <v>202875.4</v>
       </c>
       <c r="N2" s="116"/>
     </row>
@@ -14170,7 +14197,7 @@
       <c r="C3" s="26"/>
       <c r="D3" s="118" t="str">
         <f>CHOOSE(WEEKDAY(E1), "Neděle", "Pondělí", "Úterý", "Středa", "Čtvrtek", "Pátek", "Sobota")</f>
-        <v>Neděle</v>
+        <v>Pondělí</v>
       </c>
       <c r="E3" s="10"/>
       <c r="H3" s="20"/>
@@ -14179,7 +14206,7 @@
         <v>590</v>
       </c>
       <c r="M3" s="120">
-        <v>51342.0</v>
+        <v>103527.0</v>
       </c>
       <c r="N3" s="116"/>
     </row>
@@ -14199,7 +14226,7 @@
         <v>591</v>
       </c>
       <c r="M4" s="120">
-        <v>51506.0</v>
+        <v>106114.0</v>
       </c>
       <c r="N4" s="116"/>
     </row>
@@ -14223,7 +14250,7 @@
         <v>593</v>
       </c>
       <c r="M5" s="120">
-        <v>33154.0</v>
+        <v>77921.90000000001</v>
       </c>
       <c r="N5" s="116"/>
     </row>
@@ -14243,7 +14270,7 @@
         <v>594</v>
       </c>
       <c r="M6" s="120">
-        <v>1314.0</v>
+        <v>6797.0</v>
       </c>
       <c r="N6" s="116"/>
     </row>
@@ -14251,14 +14278,14 @@
       <c r="A7" s="125"/>
       <c r="B7" s="126">
         <f>TEXT(SUMPRODUCT((IFERROR(LEFT(D10:D30, FIND(":", D10:D30) - 1) * 60, 0) + IFERROR(MID(D10:D30, FIND(":", D10:D30) + 1, LEN(D10:D30) - FIND(":", D10:D30)), 0))), "[h]:mm")/60</f>
-        <v>145</v>
+        <v>292.5</v>
       </c>
       <c r="C7" s="27"/>
       <c r="D7" s="27"/>
       <c r="E7" s="18"/>
       <c r="F7" s="127">
         <f>TEXT(SUMPRODUCT((IFERROR(LEFT(H10:H30, FIND(":", H10:H30) - 1) * 60, 0) + IFERROR(MID(H10:H30, FIND(":", H10:H30) + 1, LEN(H10:H30) - FIND(":", H10:H30)), 0))), "[h]:mm")/60</f>
-        <v>69</v>
+        <v>147</v>
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
@@ -14322,14 +14349,14 @@
         <v>618</v>
       </c>
       <c r="J9" s="141">
-        <v>-1937.0</v>
+        <v>4.499999999989086</v>
       </c>
       <c r="K9" s="10"/>
       <c r="L9" s="142" t="s">
         <v>597</v>
       </c>
       <c r="M9" s="120">
-        <v>24234.0</v>
+        <v>44490.0</v>
       </c>
       <c r="N9" s="116"/>
     </row>
@@ -14339,7 +14366,7 @@
         <v>635</v>
       </c>
       <c r="C10" s="145">
-        <v>5.0</v>
+        <v>7.0</v>
       </c>
       <c r="D10" s="145" t="s">
         <v>636</v>
@@ -14351,13 +14378,13 @@
         <v>638</v>
       </c>
       <c r="G10" s="145">
-        <v>5.0</v>
+        <v>9.0</v>
       </c>
       <c r="H10" s="145" t="s">
         <v>639</v>
       </c>
       <c r="I10" s="147">
-        <v>32.0</v>
+        <v>77.0</v>
       </c>
       <c r="J10" s="35"/>
       <c r="K10" s="20"/>
@@ -14375,25 +14402,25 @@
         <v>640</v>
       </c>
       <c r="C11" s="145">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
       <c r="D11" s="145" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="E11" s="146" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="F11" s="144" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="G11" s="145">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="H11" s="145" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="I11" s="147">
-        <v>3.0</v>
+        <v>7.0</v>
       </c>
       <c r="J11" s="35"/>
       <c r="K11" s="20"/>
@@ -14401,28 +14428,36 @@
         <v>596</v>
       </c>
       <c r="M11" s="149">
-        <v>6262.0</v>
+        <v>21730.0</v>
       </c>
       <c r="N11" s="116"/>
     </row>
     <row r="12" ht="18.75" customHeight="1">
       <c r="A12" s="143"/>
       <c r="B12" s="144" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C12" s="145">
-        <v>6.0</v>
+        <v>12.0</v>
       </c>
       <c r="D12" s="145" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E12" s="146" t="s">
-        <v>646</v>
-      </c>
-      <c r="F12" s="144"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="147"/>
+        <v>647</v>
+      </c>
+      <c r="F12" s="144" t="s">
+        <v>648</v>
+      </c>
+      <c r="G12" s="145">
+        <v>1.0</v>
+      </c>
+      <c r="H12" s="145" t="s">
+        <v>649</v>
+      </c>
+      <c r="I12" s="147">
+        <v>3.0</v>
+      </c>
       <c r="J12" s="35"/>
       <c r="K12" s="20"/>
       <c r="L12" s="150" t="s">
@@ -14433,11 +14468,17 @@
     </row>
     <row r="13" ht="18.75" customHeight="1">
       <c r="A13" s="143"/>
-      <c r="B13" s="144"/>
-      <c r="C13" s="145"/>
-      <c r="D13" s="145"/>
+      <c r="B13" s="144" t="s">
+        <v>650</v>
+      </c>
+      <c r="C13" s="145">
+        <v>3.0</v>
+      </c>
+      <c r="D13" s="145" t="s">
+        <v>651</v>
+      </c>
       <c r="E13" s="146" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="F13" s="144"/>
       <c r="G13" s="145"/>
@@ -14455,11 +14496,17 @@
     </row>
     <row r="14" ht="18.75" customHeight="1">
       <c r="A14" s="143"/>
-      <c r="B14" s="144"/>
-      <c r="C14" s="145"/>
-      <c r="D14" s="145"/>
+      <c r="B14" s="144" t="s">
+        <v>652</v>
+      </c>
+      <c r="C14" s="145">
+        <v>1.0</v>
+      </c>
+      <c r="D14" s="145" t="s">
+        <v>653</v>
+      </c>
       <c r="E14" s="146" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="F14" s="144"/>
       <c r="G14" s="145"/>
@@ -14477,11 +14524,17 @@
     </row>
     <row r="15" ht="18.75" customHeight="1">
       <c r="A15" s="143"/>
-      <c r="B15" s="144"/>
-      <c r="C15" s="145"/>
-      <c r="D15" s="145"/>
+      <c r="B15" s="144" t="s">
+        <v>654</v>
+      </c>
+      <c r="C15" s="145">
+        <v>1.0</v>
+      </c>
+      <c r="D15" s="145" t="s">
+        <v>655</v>
+      </c>
       <c r="E15" s="146" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="F15" s="144"/>
       <c r="G15" s="145"/>
@@ -14493,15 +14546,21 @@
         <v>610</v>
       </c>
       <c r="M15" s="120">
-        <v>0.0</v>
+        <v>71.0</v>
       </c>
       <c r="N15" s="116"/>
     </row>
     <row r="16" ht="18.75" customHeight="1">
       <c r="A16" s="143"/>
-      <c r="B16" s="144"/>
-      <c r="C16" s="145"/>
-      <c r="D16" s="145"/>
+      <c r="B16" s="144" t="s">
+        <v>656</v>
+      </c>
+      <c r="C16" s="145">
+        <v>1.0</v>
+      </c>
+      <c r="D16" s="145" t="s">
+        <v>653</v>
+      </c>
       <c r="E16" s="152"/>
       <c r="F16" s="144"/>
       <c r="G16" s="145"/>
@@ -14513,7 +14572,7 @@
         <v>611</v>
       </c>
       <c r="M16" s="120">
-        <v>863.0</v>
+        <v>1647.0</v>
       </c>
       <c r="N16" s="116"/>
     </row>
@@ -14533,7 +14592,7 @@
         <v>612</v>
       </c>
       <c r="M17" s="154">
-        <v>1095.0</v>
+        <v>3280.0</v>
       </c>
       <c r="N17" s="116"/>
     </row>
@@ -14604,16 +14663,16 @@
       <c r="H21" s="145"/>
       <c r="I21" s="147"/>
       <c r="J21" s="164">
-        <v>8.0</v>
+        <v>19.0</v>
       </c>
       <c r="K21" s="165">
-        <v>2838.0</v>
+        <v>8428.0</v>
       </c>
       <c r="L21" s="166">
-        <v>5.0</v>
+        <v>24.0</v>
       </c>
       <c r="M21" s="167" t="s">
-        <v>648</v>
+        <v>657</v>
       </c>
       <c r="N21" s="156"/>
     </row>
@@ -14668,16 +14727,16 @@
       <c r="H24" s="145"/>
       <c r="I24" s="147"/>
       <c r="J24" s="172">
-        <v>5.0</v>
+        <v>11.0</v>
       </c>
       <c r="K24" s="166">
-        <v>655.0</v>
+        <v>1363.0</v>
       </c>
       <c r="L24" s="166">
-        <v>65.0</v>
+        <v>169.0</v>
       </c>
       <c r="M24" s="173">
-        <v>3.0</v>
+        <v>21.0</v>
       </c>
       <c r="N24" s="156"/>
     </row>
@@ -14730,14 +14789,14 @@
       <c r="H27" s="145"/>
       <c r="I27" s="147"/>
       <c r="J27" s="178">
-        <v>2.0</v>
+        <v>11.0</v>
       </c>
       <c r="K27" s="94"/>
       <c r="L27" s="179">
-        <v>0.0821969696969697</v>
+        <v>0.12405159314875214</v>
       </c>
       <c r="M27" s="180">
-        <v>2.0</v>
+        <v>13.0</v>
       </c>
       <c r="N27" s="156"/>
     </row>
@@ -14788,10 +14847,10 @@
       <c r="J30" s="17"/>
       <c r="K30" s="27"/>
       <c r="L30" s="183">
-        <v>0.9178030303030302</v>
+        <v>0.8759484068512479</v>
       </c>
       <c r="M30" s="184">
-        <v>0.03636363636363636</v>
+        <v>0.06908715639365795</v>
       </c>
       <c r="N30" s="156"/>
     </row>
@@ -14937,7 +14996,7 @@
       <c r="B3" s="4"/>
       <c r="C3" s="186"/>
       <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
+      <c r="E3" s="185"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -14971,7 +15030,7 @@
       <c r="B4" s="4"/>
       <c r="C4" s="186"/>
       <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
+      <c r="E4" s="185"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -15005,7 +15064,7 @@
       <c r="B5" s="186"/>
       <c r="C5" s="186"/>
       <c r="D5" s="4"/>
-      <c r="E5" s="185"/>
+      <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -15072,13 +15131,13 @@
       <c r="B7" s="4"/>
       <c r="C7" s="186"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="185"/>
+      <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
-      <c r="K7" s="185"/>
+      <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
@@ -15097,6 +15156,7 @@
       <c r="AA7" s="185"/>
       <c r="AB7" s="185"/>
       <c r="AC7" s="185"/>
+      <c r="AD7" s="185"/>
       <c r="AE7" s="185"/>
       <c r="AF7" s="185"/>
     </row>
@@ -15179,7 +15239,7 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
-      <c r="K10" s="185"/>
+      <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
@@ -15246,7 +15306,7 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
+      <c r="K12" s="185"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
@@ -15376,7 +15436,7 @@
       <c r="B16" s="4"/>
       <c r="C16" s="186"/>
       <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="E16" s="185"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -15410,7 +15470,7 @@
       <c r="B17" s="186"/>
       <c r="C17" s="186"/>
       <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="E17" s="185"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -15444,7 +15504,7 @@
       <c r="B18" s="186"/>
       <c r="C18" s="186"/>
       <c r="D18" s="4"/>
-      <c r="E18" s="185"/>
+      <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -15512,7 +15572,7 @@
       <c r="B20" s="4"/>
       <c r="C20" s="186"/>
       <c r="D20" s="4"/>
-      <c r="E20" s="185"/>
+      <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -15654,7 +15714,7 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="185"/>
+      <c r="K24" s="4"/>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
@@ -15682,7 +15742,7 @@
       <c r="B25" s="186"/>
       <c r="C25" s="186"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
+      <c r="E25" s="185"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -15716,7 +15776,7 @@
       <c r="B26" s="4"/>
       <c r="C26" s="186"/>
       <c r="D26" s="4"/>
-      <c r="E26" s="185"/>
+      <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -15755,7 +15815,7 @@
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
-      <c r="K27" s="185"/>
+      <c r="K27" s="4"/>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
@@ -15783,7 +15843,7 @@
       <c r="B28" s="186"/>
       <c r="C28" s="186"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="E28" s="185"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -15817,7 +15877,7 @@
       <c r="B29" s="186"/>
       <c r="C29" s="186"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="185"/>
+      <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -15919,13 +15979,13 @@
       <c r="B32" s="4"/>
       <c r="C32" s="186"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="E32" s="185"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
+      <c r="K32" s="185"/>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
@@ -15959,7 +16019,7 @@
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
-      <c r="K33" s="185"/>
+      <c r="K33" s="4"/>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
@@ -16027,7 +16087,7 @@
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
-      <c r="K35" s="185"/>
+      <c r="K35" s="4"/>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
       <c r="N35" s="4"/>
@@ -16061,7 +16121,7 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
+      <c r="K36" s="185"/>
       <c r="L36" s="4"/>
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
@@ -16089,7 +16149,7 @@
       <c r="B37" s="4"/>
       <c r="C37" s="186"/>
       <c r="D37" s="4"/>
-      <c r="E37" s="185"/>
+      <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -16129,7 +16189,7 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
-      <c r="K38" s="4"/>
+      <c r="K38" s="185"/>
       <c r="L38" s="4"/>
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
@@ -16197,7 +16257,7 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="185"/>
+      <c r="K40" s="4"/>
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
@@ -16264,7 +16324,7 @@
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
-      <c r="K42" s="185"/>
+      <c r="K42" s="4"/>
       <c r="L42" s="4"/>
       <c r="M42" s="4"/>
       <c r="N42" s="4"/>
@@ -16394,7 +16454,7 @@
       <c r="B46" s="4"/>
       <c r="C46" s="186"/>
       <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="E46" s="185"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -16468,7 +16528,7 @@
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
       <c r="J48" s="4"/>
-      <c r="K48" s="4"/>
+      <c r="K48" s="185"/>
       <c r="L48" s="4"/>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
@@ -16564,7 +16624,7 @@
       <c r="B51" s="4"/>
       <c r="C51" s="186"/>
       <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
+      <c r="E51" s="185"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -16598,7 +16658,7 @@
       <c r="B52" s="186"/>
       <c r="C52" s="186"/>
       <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
+      <c r="E52" s="185"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -16632,7 +16692,7 @@
       <c r="B53" s="4"/>
       <c r="C53" s="186"/>
       <c r="D53" s="4"/>
-      <c r="E53" s="185"/>
+      <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -16666,7 +16726,7 @@
       <c r="B54" s="4"/>
       <c r="C54" s="186"/>
       <c r="D54" s="4"/>
-      <c r="E54" s="185"/>
+      <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -16700,7 +16760,7 @@
       <c r="B55" s="4"/>
       <c r="C55" s="186"/>
       <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
+      <c r="E55" s="185"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -16734,13 +16794,13 @@
       <c r="B56" s="4"/>
       <c r="C56" s="186"/>
       <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
+      <c r="E56" s="185"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
+      <c r="K56" s="185"/>
       <c r="L56" s="4"/>
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
@@ -16798,22 +16858,22 @@
       <c r="AF57" s="185"/>
     </row>
     <row r="58">
-      <c r="A58" s="185"/>
-      <c r="B58" s="185"/>
-      <c r="C58" s="187"/>
-      <c r="D58" s="185"/>
-      <c r="E58" s="185"/>
-      <c r="F58" s="185"/>
-      <c r="G58" s="185"/>
-      <c r="H58" s="185"/>
-      <c r="I58" s="185"/>
-      <c r="J58" s="185"/>
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="186"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
       <c r="K58" s="185"/>
-      <c r="L58" s="185"/>
-      <c r="M58" s="185"/>
-      <c r="N58" s="185"/>
-      <c r="O58" s="185"/>
-      <c r="P58" s="185"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="4"/>
       <c r="Q58" s="185"/>
       <c r="R58" s="185"/>
       <c r="S58" s="185"/>
@@ -16832,22 +16892,22 @@
       <c r="AF58" s="185"/>
     </row>
     <row r="59">
-      <c r="A59" s="185"/>
-      <c r="B59" s="185"/>
-      <c r="C59" s="187"/>
-      <c r="D59" s="185"/>
-      <c r="E59" s="185"/>
-      <c r="F59" s="185"/>
-      <c r="G59" s="185"/>
-      <c r="H59" s="185"/>
-      <c r="I59" s="185"/>
-      <c r="J59" s="185"/>
-      <c r="K59" s="185"/>
-      <c r="L59" s="185"/>
-      <c r="M59" s="185"/>
-      <c r="N59" s="185"/>
-      <c r="O59" s="185"/>
-      <c r="P59" s="185"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="186"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4"/>
+      <c r="I59" s="4"/>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4"/>
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
+      <c r="P59" s="4"/>
       <c r="Q59" s="185"/>
       <c r="R59" s="185"/>
       <c r="S59" s="185"/>
@@ -16866,22 +16926,22 @@
       <c r="AF59" s="185"/>
     </row>
     <row r="60">
-      <c r="A60" s="185"/>
-      <c r="B60" s="185"/>
-      <c r="C60" s="187"/>
-      <c r="D60" s="185"/>
-      <c r="E60" s="185"/>
-      <c r="F60" s="185"/>
-      <c r="G60" s="185"/>
-      <c r="H60" s="185"/>
-      <c r="I60" s="185"/>
-      <c r="J60" s="185"/>
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="186"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
       <c r="K60" s="185"/>
-      <c r="L60" s="185"/>
-      <c r="M60" s="185"/>
-      <c r="N60" s="185"/>
-      <c r="O60" s="185"/>
-      <c r="P60" s="185"/>
+      <c r="L60" s="4"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="4"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="4"/>
       <c r="Q60" s="185"/>
       <c r="R60" s="185"/>
       <c r="S60" s="185"/>
@@ -16900,22 +16960,22 @@
       <c r="AF60" s="185"/>
     </row>
     <row r="61">
-      <c r="A61" s="185"/>
-      <c r="B61" s="185"/>
-      <c r="C61" s="187"/>
-      <c r="D61" s="185"/>
-      <c r="E61" s="185"/>
-      <c r="F61" s="185"/>
-      <c r="G61" s="185"/>
-      <c r="H61" s="185"/>
-      <c r="I61" s="185"/>
-      <c r="J61" s="185"/>
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="186"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="4"/>
+      <c r="H61" s="4"/>
+      <c r="I61" s="4"/>
+      <c r="J61" s="4"/>
       <c r="K61" s="185"/>
-      <c r="L61" s="185"/>
-      <c r="M61" s="185"/>
-      <c r="N61" s="185"/>
-      <c r="O61" s="185"/>
-      <c r="P61" s="185"/>
+      <c r="L61" s="4"/>
+      <c r="M61" s="4"/>
+      <c r="N61" s="4"/>
+      <c r="O61" s="4"/>
+      <c r="P61" s="4"/>
       <c r="Q61" s="185"/>
       <c r="R61" s="185"/>
       <c r="S61" s="185"/>
@@ -16934,22 +16994,22 @@
       <c r="AF61" s="185"/>
     </row>
     <row r="62">
-      <c r="A62" s="185"/>
-      <c r="B62" s="185"/>
-      <c r="C62" s="187"/>
-      <c r="D62" s="185"/>
-      <c r="E62" s="185"/>
-      <c r="F62" s="185"/>
-      <c r="G62" s="185"/>
-      <c r="H62" s="185"/>
-      <c r="I62" s="185"/>
-      <c r="J62" s="185"/>
+      <c r="A62" s="4"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="186"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
       <c r="K62" s="185"/>
-      <c r="L62" s="185"/>
-      <c r="M62" s="185"/>
-      <c r="N62" s="185"/>
-      <c r="O62" s="185"/>
-      <c r="P62" s="185"/>
+      <c r="L62" s="4"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="4"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="4"/>
       <c r="Q62" s="185"/>
       <c r="R62" s="185"/>
       <c r="S62" s="185"/>
@@ -16968,22 +17028,22 @@
       <c r="AF62" s="185"/>
     </row>
     <row r="63">
-      <c r="A63" s="185"/>
-      <c r="B63" s="185"/>
-      <c r="C63" s="187"/>
-      <c r="D63" s="185"/>
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="186"/>
+      <c r="D63" s="4"/>
       <c r="E63" s="185"/>
-      <c r="F63" s="185"/>
-      <c r="G63" s="185"/>
-      <c r="H63" s="185"/>
-      <c r="I63" s="185"/>
-      <c r="J63" s="185"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
       <c r="K63" s="185"/>
-      <c r="L63" s="185"/>
-      <c r="M63" s="185"/>
-      <c r="N63" s="185"/>
-      <c r="O63" s="185"/>
-      <c r="P63" s="185"/>
+      <c r="L63" s="4"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="4"/>
+      <c r="O63" s="4"/>
+      <c r="P63" s="4"/>
       <c r="Q63" s="185"/>
       <c r="R63" s="185"/>
       <c r="S63" s="185"/>
@@ -17002,22 +17062,22 @@
       <c r="AF63" s="185"/>
     </row>
     <row r="64">
-      <c r="A64" s="185"/>
-      <c r="B64" s="185"/>
-      <c r="C64" s="187"/>
-      <c r="D64" s="185"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="186"/>
+      <c r="D64" s="4"/>
       <c r="E64" s="185"/>
-      <c r="F64" s="185"/>
-      <c r="G64" s="185"/>
-      <c r="H64" s="185"/>
-      <c r="I64" s="185"/>
-      <c r="J64" s="185"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
       <c r="K64" s="185"/>
-      <c r="L64" s="185"/>
-      <c r="M64" s="185"/>
-      <c r="N64" s="185"/>
-      <c r="O64" s="185"/>
-      <c r="P64" s="185"/>
+      <c r="L64" s="4"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="4"/>
+      <c r="O64" s="4"/>
+      <c r="P64" s="4"/>
       <c r="Q64" s="185"/>
       <c r="R64" s="185"/>
       <c r="S64" s="185"/>
@@ -17602,6 +17662,7 @@
       <c r="AA81" s="185"/>
       <c r="AB81" s="185"/>
       <c r="AC81" s="185"/>
+      <c r="AD81" s="185"/>
       <c r="AE81" s="185"/>
       <c r="AF81" s="185"/>
     </row>
@@ -18547,6 +18608,7 @@
       <c r="K110" s="185"/>
       <c r="L110" s="185"/>
       <c r="M110" s="185"/>
+      <c r="N110" s="185"/>
       <c r="O110" s="185"/>
       <c r="P110" s="185"/>
       <c r="Q110" s="185"/>
@@ -18670,9 +18732,11 @@
       <c r="K114" s="185"/>
       <c r="L114" s="185"/>
       <c r="M114" s="185"/>
+      <c r="N114" s="185"/>
       <c r="O114" s="185"/>
       <c r="P114" s="185"/>
       <c r="Q114" s="185"/>
+      <c r="R114" s="185"/>
       <c r="S114" s="185"/>
       <c r="T114" s="185"/>
       <c r="U114" s="185"/>
@@ -18681,8 +18745,10 @@
       <c r="X114" s="185"/>
       <c r="Y114" s="185"/>
       <c r="Z114" s="185"/>
+      <c r="AA114" s="185"/>
       <c r="AB114" s="185"/>
       <c r="AC114" s="185"/>
+      <c r="AD114" s="185"/>
       <c r="AE114" s="185"/>
       <c r="AF114" s="185"/>
     </row>
@@ -18700,6 +18766,7 @@
       <c r="K115" s="185"/>
       <c r="L115" s="185"/>
       <c r="M115" s="185"/>
+      <c r="N115" s="185"/>
       <c r="O115" s="185"/>
       <c r="P115" s="185"/>
       <c r="Q115" s="185"/>
@@ -18730,9 +18797,11 @@
       <c r="K116" s="185"/>
       <c r="L116" s="185"/>
       <c r="M116" s="185"/>
+      <c r="N116" s="185"/>
       <c r="O116" s="185"/>
       <c r="P116" s="185"/>
       <c r="Q116" s="185"/>
+      <c r="R116" s="185"/>
       <c r="S116" s="185"/>
       <c r="T116" s="185"/>
       <c r="U116" s="185"/>
@@ -18741,6 +18810,7 @@
       <c r="X116" s="185"/>
       <c r="Y116" s="185"/>
       <c r="Z116" s="185"/>
+      <c r="AA116" s="185"/>
       <c r="AB116" s="185"/>
       <c r="AC116" s="185"/>
       <c r="AE116" s="185"/>
@@ -18764,6 +18834,7 @@
       <c r="O117" s="185"/>
       <c r="P117" s="185"/>
       <c r="Q117" s="185"/>
+      <c r="R117" s="185"/>
       <c r="S117" s="185"/>
       <c r="T117" s="185"/>
       <c r="U117" s="185"/>
@@ -18772,6 +18843,7 @@
       <c r="X117" s="185"/>
       <c r="Y117" s="185"/>
       <c r="Z117" s="185"/>
+      <c r="AA117" s="185"/>
       <c r="AB117" s="185"/>
       <c r="AC117" s="185"/>
       <c r="AE117" s="185"/>
@@ -18791,9 +18863,11 @@
       <c r="K118" s="185"/>
       <c r="L118" s="185"/>
       <c r="M118" s="185"/>
+      <c r="N118" s="185"/>
       <c r="O118" s="185"/>
       <c r="P118" s="185"/>
       <c r="Q118" s="185"/>
+      <c r="R118" s="185"/>
       <c r="S118" s="185"/>
       <c r="T118" s="185"/>
       <c r="U118" s="185"/>
@@ -18802,6 +18876,7 @@
       <c r="X118" s="185"/>
       <c r="Y118" s="185"/>
       <c r="Z118" s="185"/>
+      <c r="AA118" s="185"/>
       <c r="AB118" s="185"/>
       <c r="AC118" s="185"/>
       <c r="AE118" s="185"/>
@@ -18821,6 +18896,7 @@
       <c r="K119" s="185"/>
       <c r="L119" s="185"/>
       <c r="M119" s="185"/>
+      <c r="N119" s="185"/>
       <c r="O119" s="185"/>
       <c r="P119" s="185"/>
       <c r="Q119" s="185"/>
@@ -18851,6 +18927,7 @@
       <c r="K120" s="185"/>
       <c r="L120" s="185"/>
       <c r="M120" s="185"/>
+      <c r="N120" s="185"/>
       <c r="O120" s="185"/>
       <c r="P120" s="185"/>
       <c r="Q120" s="185"/>
@@ -19166,10 +19243,10 @@
     </row>
     <row r="4">
       <c r="A4" s="191" t="s">
-        <v>649</v>
+        <v>658</v>
       </c>
       <c r="B4" s="191" t="s">
-        <v>650</v>
+        <v>659</v>
       </c>
       <c r="C4" s="2" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Manažer")</f>
@@ -19440,8 +19517,8 @@
         <v>Malešice</v>
       </c>
       <c r="G8" s="2" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Chodov")</f>
-        <v>Chodov</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Zličín")</f>
+        <v>Zličín</v>
       </c>
       <c r="H8" s="2" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Prosek")</f>
@@ -19802,7 +19879,7 @@
       </c>
       <c r="B14" s="192" t="str">
         <f>IF(OR(E14=Report!$B$1, F14=Report!$B$1, G14=Report!$B$1, H14=Report!$B$1), D14, "")</f>
-        <v/>
+        <v>Coufal Jakub</v>
       </c>
       <c r="C14" s="2" t="b">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
@@ -19820,7 +19897,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Malešice")</f>
         <v>Malešice</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Prosek")</f>
+        <v>Prosek</v>
+      </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -20840,7 +20920,7 @@
       </c>
       <c r="B31" s="192" t="str">
         <f>IF(OR(E31=Report!$B$1, F31=Report!$B$1, G31=Report!$B$1, H31=Report!$B$1), D31, "")</f>
-        <v/>
+        <v>Gorol Patrik</v>
       </c>
       <c r="C31" s="2" t="b">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
@@ -20858,7 +20938,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Libuš")</f>
         <v>Libuš</v>
       </c>
-      <c r="G31" s="2"/>
+      <c r="G31" s="2" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Prosek")</f>
+        <v>Prosek</v>
+      </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
@@ -23925,7 +24008,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Malešice")</f>
         <v>Malešice</v>
       </c>
-      <c r="H89" s="2"/>
+      <c r="H89" s="2" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Výroba")</f>
+        <v>Výroba</v>
+      </c>
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
       <c r="K89" s="2"/>
@@ -26009,8 +26095,14 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D126" s="2"/>
-      <c r="E126" s="2"/>
+      <c r="D126" s="2" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pavel Břicháč")</f>
+        <v>Pavel Břicháč</v>
+      </c>
+      <c r="E126" s="2" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Libuš")</f>
+        <v>Libuš</v>
+      </c>
       <c r="F126" s="2"/>
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
@@ -26028,8 +26120,8 @@
       <c r="T126" s="2"/>
       <c r="U126" s="2"/>
       <c r="V126" s="190">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),231.474)</f>
+        <v>231.474</v>
       </c>
       <c r="W126" s="190">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -60944,7 +61036,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="194" t="s">
-        <v>651</v>
+        <v>660</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -60976,28 +61068,28 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>652</v>
+        <v>661</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>654</v>
+        <v>663</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>655</v>
+        <v>664</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>656</v>
+        <v>665</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>657</v>
+        <v>666</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>658</v>
+        <v>667</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>659</v>
+        <v>668</v>
       </c>
       <c r="I2" s="185"/>
       <c r="J2" s="185"/>
@@ -61026,22 +61118,22 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>660</v>
+        <v>669</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>661</v>
+        <v>670</v>
       </c>
       <c r="C3" s="185"/>
       <c r="D3" s="185"/>
       <c r="E3" s="4" t="s">
-        <v>661</v>
+        <v>670</v>
       </c>
       <c r="F3" s="185"/>
       <c r="G3" s="4" t="s">
-        <v>662</v>
+        <v>671</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>663</v>
+        <v>672</v>
       </c>
       <c r="I3" s="185"/>
       <c r="J3" s="185"/>
@@ -61063,20 +61155,20 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>664</v>
+        <v>673</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>665</v>
+        <v>674</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>665</v>
+        <v>674</v>
       </c>
       <c r="D4" s="185"/>
       <c r="E4" s="4" t="s">
-        <v>666</v>
+        <v>675</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>667</v>
+        <v>676</v>
       </c>
       <c r="G4" s="185"/>
       <c r="H4" s="185"/>
@@ -61100,18 +61192,18 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>668</v>
+        <v>677</v>
       </c>
       <c r="B5" s="185"/>
       <c r="C5" s="4" t="s">
-        <v>661</v>
+        <v>670</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>661</v>
+        <v>670</v>
       </c>
       <c r="E5" s="185"/>
       <c r="F5" s="4" t="s">
-        <v>662</v>
+        <v>671</v>
       </c>
       <c r="G5" s="185"/>
       <c r="H5" s="185"/>
@@ -61138,15 +61230,15 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>669</v>
+        <v>678</v>
       </c>
       <c r="C6" s="185"/>
       <c r="D6" s="4" t="s">
-        <v>666</v>
+        <v>675</v>
       </c>
       <c r="E6" s="185"/>
       <c r="F6" s="4" t="s">
-        <v>666</v>
+        <v>675</v>
       </c>
       <c r="G6" s="185"/>
       <c r="H6" s="185"/>
@@ -61173,14 +61265,14 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>670</v>
+        <v>679</v>
       </c>
       <c r="C7" s="185"/>
       <c r="D7" s="4" t="s">
-        <v>671</v>
+        <v>680</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>671</v>
+        <v>680</v>
       </c>
       <c r="G7" s="185"/>
       <c r="I7" s="185"/>
@@ -61204,14 +61296,14 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="s">
-        <v>672</v>
+        <v>681</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>673</v>
+        <v>682</v>
       </c>
       <c r="F8" s="185"/>
       <c r="H8" s="4" t="s">
-        <v>673</v>
+        <v>682</v>
       </c>
       <c r="I8" s="185"/>
       <c r="J8" s="185"/>
@@ -61236,17 +61328,17 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>674</v>
+        <v>683</v>
       </c>
       <c r="D9" s="185"/>
       <c r="E9" s="4" t="s">
-        <v>675</v>
+        <v>684</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>675</v>
+        <v>684</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>675</v>
+        <v>684</v>
       </c>
       <c r="H9" s="185"/>
       <c r="I9" s="185"/>
@@ -61271,14 +61363,14 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>676</v>
+        <v>685</v>
       </c>
       <c r="F10" s="185"/>
       <c r="G10" s="4" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>678</v>
+        <v>687</v>
       </c>
       <c r="I10" s="185"/>
       <c r="J10" s="185"/>
@@ -61491,7 +61583,7 @@
       <c r="Y19" s="185"/>
       <c r="Z19" s="185"/>
       <c r="AA19" s="4" t="s">
-        <v>679</v>
+        <v>688</v>
       </c>
       <c r="AB19" s="4">
         <v>-11.0</v>
@@ -61816,7 +61908,7 @@
       <c r="Y30" s="185"/>
       <c r="Z30" s="185"/>
       <c r="AA30" s="4" t="s">
-        <v>680</v>
+        <v>689</v>
       </c>
       <c r="AB30" s="4">
         <v>-8.0</v>
@@ -61937,7 +62029,7 @@
       <c r="Y34" s="185"/>
       <c r="Z34" s="185"/>
       <c r="AA34" s="4" t="s">
-        <v>681</v>
+        <v>690</v>
       </c>
       <c r="AB34" s="4">
         <v>0.0</v>
@@ -62056,7 +62148,7 @@
       <c r="Y38" s="185"/>
       <c r="Z38" s="185"/>
       <c r="AA38" s="4" t="s">
-        <v>682</v>
+        <v>691</v>
       </c>
       <c r="AB38" s="4">
         <v>-12.0</v>
@@ -62090,7 +62182,7 @@
       <c r="Y39" s="185"/>
       <c r="Z39" s="185"/>
       <c r="AA39" s="4" t="s">
-        <v>683</v>
+        <v>692</v>
       </c>
       <c r="AB39" s="4">
         <v>0.0</v>
@@ -62182,7 +62274,7 @@
       <c r="Y42" s="185"/>
       <c r="Z42" s="185"/>
       <c r="AA42" s="4" t="s">
-        <v>684</v>
+        <v>693</v>
       </c>
       <c r="AB42" s="4">
         <v>6.0</v>
@@ -62361,7 +62453,7 @@
       <c r="Y48" s="185"/>
       <c r="Z48" s="185"/>
       <c r="AA48" s="4" t="s">
-        <v>685</v>
+        <v>694</v>
       </c>
       <c r="AB48" s="4">
         <v>-13.0</v>
@@ -62482,7 +62574,7 @@
       <c r="Y52" s="185"/>
       <c r="Z52" s="185"/>
       <c r="AA52" s="4" t="s">
-        <v>686</v>
+        <v>695</v>
       </c>
       <c r="AB52" s="4">
         <v>5.0</v>
@@ -62690,7 +62782,7 @@
       <c r="Y59" s="185"/>
       <c r="Z59" s="185"/>
       <c r="AA59" s="4" t="s">
-        <v>687</v>
+        <v>696</v>
       </c>
       <c r="AB59" s="4">
         <v>-9.0</v>
@@ -62811,7 +62903,7 @@
       <c r="Y63" s="185"/>
       <c r="Z63" s="185"/>
       <c r="AA63" s="4" t="s">
-        <v>688</v>
+        <v>697</v>
       </c>
       <c r="AB63" s="4">
         <v>-19.0</v>
@@ -63019,7 +63111,7 @@
       <c r="Y70" s="185"/>
       <c r="Z70" s="185"/>
       <c r="AA70" s="4" t="s">
-        <v>689</v>
+        <v>698</v>
       </c>
       <c r="AB70" s="4">
         <v>-14.0</v>
@@ -63488,7 +63580,7 @@
       <c r="Y86" s="185"/>
       <c r="Z86" s="185"/>
       <c r="AA86" s="4" t="s">
-        <v>690</v>
+        <v>699</v>
       </c>
       <c r="AB86" s="4">
         <v>-21.0</v>
@@ -63522,7 +63614,7 @@
       <c r="Y87" s="185"/>
       <c r="Z87" s="185"/>
       <c r="AA87" s="4" t="s">
-        <v>691</v>
+        <v>700</v>
       </c>
       <c r="AB87" s="4">
         <v>-7.0</v>
@@ -63556,7 +63648,7 @@
       <c r="Y88" s="185"/>
       <c r="Z88" s="185"/>
       <c r="AA88" s="4" t="s">
-        <v>692</v>
+        <v>701</v>
       </c>
       <c r="AB88" s="4">
         <v>-10.0</v>
@@ -63590,7 +63682,7 @@
       <c r="Y89" s="185"/>
       <c r="Z89" s="185"/>
       <c r="AA89" s="4" t="s">
-        <v>693</v>
+        <v>702</v>
       </c>
       <c r="AB89" s="4">
         <v>-6.0</v>
@@ -63683,7 +63775,7 @@
       <c r="Y92" s="185"/>
       <c r="Z92" s="185"/>
       <c r="AA92" s="4" t="s">
-        <v>694</v>
+        <v>703</v>
       </c>
       <c r="AB92" s="4">
         <v>-17.0</v>
@@ -63949,7 +64041,7 @@
       <c r="Y101" s="185"/>
       <c r="Z101" s="185"/>
       <c r="AA101" s="4" t="s">
-        <v>695</v>
+        <v>704</v>
       </c>
       <c r="AB101" s="4">
         <v>-6.0</v>
@@ -63983,7 +64075,7 @@
       <c r="Y102" s="185"/>
       <c r="Z102" s="185"/>
       <c r="AA102" s="4" t="s">
-        <v>696</v>
+        <v>705</v>
       </c>
       <c r="AB102" s="4">
         <v>1.0</v>
@@ -64075,7 +64167,7 @@
       <c r="Y105" s="185"/>
       <c r="Z105" s="185"/>
       <c r="AA105" s="4" t="s">
-        <v>697</v>
+        <v>706</v>
       </c>
       <c r="AB105" s="4">
         <v>-2.0</v>
@@ -64138,7 +64230,7 @@
       <c r="Y107" s="185"/>
       <c r="Z107" s="185"/>
       <c r="AA107" s="4" t="s">
-        <v>698</v>
+        <v>707</v>
       </c>
       <c r="AB107" s="4">
         <v>-12.0</v>
@@ -64230,7 +64322,7 @@
       <c r="Y110" s="185"/>
       <c r="Z110" s="185"/>
       <c r="AA110" s="4" t="s">
-        <v>699</v>
+        <v>708</v>
       </c>
       <c r="AB110" s="4">
         <v>-14.0</v>
@@ -64264,7 +64356,7 @@
       <c r="Y111" s="185"/>
       <c r="Z111" s="185"/>
       <c r="AA111" s="4" t="s">
-        <v>700</v>
+        <v>709</v>
       </c>
       <c r="AB111" s="4">
         <v>-6.0</v>
@@ -64298,7 +64390,7 @@
       <c r="Y112" s="185"/>
       <c r="Z112" s="185"/>
       <c r="AA112" s="4" t="s">
-        <v>701</v>
+        <v>710</v>
       </c>
       <c r="AB112" s="4">
         <v>-11.0</v>
@@ -64361,7 +64453,7 @@
       <c r="Y114" s="185"/>
       <c r="Z114" s="185"/>
       <c r="AA114" s="4" t="s">
-        <v>702</v>
+        <v>711</v>
       </c>
       <c r="AB114" s="4">
         <v>-1.0</v>
@@ -64453,7 +64545,7 @@
       <c r="Y117" s="185"/>
       <c r="Z117" s="185"/>
       <c r="AA117" s="4" t="s">
-        <v>703</v>
+        <v>712</v>
       </c>
       <c r="AB117" s="4">
         <v>12.0</v>
@@ -64516,7 +64608,7 @@
       <c r="Y119" s="185"/>
       <c r="Z119" s="185"/>
       <c r="AA119" s="4" t="s">
-        <v>704</v>
+        <v>713</v>
       </c>
       <c r="AB119" s="4">
         <v>-17.0</v>
@@ -64637,7 +64729,7 @@
       <c r="Y123" s="185"/>
       <c r="Z123" s="185"/>
       <c r="AA123" s="4" t="s">
-        <v>705</v>
+        <v>714</v>
       </c>
       <c r="AB123" s="4">
         <v>-15.0</v>
@@ -64788,7 +64880,7 @@
       <c r="Y128" s="185"/>
       <c r="Z128" s="185"/>
       <c r="AA128" s="4" t="s">
-        <v>706</v>
+        <v>715</v>
       </c>
       <c r="AB128" s="4">
         <v>-11.0</v>
@@ -65173,7 +65265,7 @@
       <c r="Y141" s="185"/>
       <c r="Z141" s="185"/>
       <c r="AA141" s="4" t="s">
-        <v>707</v>
+        <v>716</v>
       </c>
       <c r="AB141" s="4">
         <v>-10.0</v>

</xml_diff>